<commit_message>
products schema change to enable recommendation for the products
</commit_message>
<xml_diff>
--- a/Frontend/src/data/Acne Serums.xlsx
+++ b/Frontend/src/data/Acne Serums.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imala\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unavarasty\FYP\Code\Web Development\AI-Powered-Skin-Care-Ecommerce\Frontend\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BB9B1A-907A-4C50-B72E-04397CE87CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590AFCEA-400D-48FB-83F6-CCD53514140C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,9 +76,6 @@
     <t>Serum</t>
   </si>
   <si>
-    <t>Active Acne</t>
-  </si>
-  <si>
     <t>2% Salicylic Acid, Ceramides, Lactic-Glycolic Acid</t>
   </si>
   <si>
@@ -194,6 +191,9 @@
   </si>
   <si>
     <t>Olim Naturals</t>
+  </si>
+  <si>
+    <t>Acne</t>
   </si>
 </sst>
 </file>
@@ -270,16 +270,15 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -647,22 +646,22 @@
         <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4">
+        <v>19</v>
+      </c>
+      <c r="F3">
         <v>19.989999999999998</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -676,22 +675,22 @@
         <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="4">
+        <v>20</v>
+      </c>
+      <c r="F4">
         <v>11.99</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -705,22 +704,22 @@
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="4">
+        <v>21</v>
+      </c>
+      <c r="F5">
         <v>39.99</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -734,22 +733,22 @@
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="4">
+        <v>22</v>
+      </c>
+      <c r="F6">
         <v>9.99</v>
       </c>
       <c r="G6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
         <v>34</v>
       </c>
-      <c r="H6" t="s">
-        <v>35</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -763,22 +762,22 @@
         <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="4">
+        <v>23</v>
+      </c>
+      <c r="F7">
         <v>22.95</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -792,22 +791,22 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="4">
+        <v>24</v>
+      </c>
+      <c r="F8">
         <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -821,22 +820,22 @@
         <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="4">
+        <v>25</v>
+      </c>
+      <c r="F9">
         <v>42</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -850,22 +849,22 @@
         <v>17</v>
       </c>
       <c r="D10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" t="s">
         <v>18</v>
       </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="4">
+      <c r="F10">
         <v>19.989999999999998</v>
       </c>
       <c r="G10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -873,28 +872,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
         <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F11">
         <v>15</v>
       </c>
       <c r="G11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="H11" t="s">
-        <v>37</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -902,28 +901,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" t="s">
         <v>50</v>
-      </c>
-      <c r="C12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" t="s">
-        <v>51</v>
       </c>
       <c r="F12">
         <v>7</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="H12" t="s">
-        <v>37</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -931,28 +930,28 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" t="s">
         <v>54</v>
-      </c>
-      <c r="C13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" t="s">
-        <v>55</v>
       </c>
       <c r="F13">
         <v>5</v>
       </c>
       <c r="G13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>